<commit_message>
Add Run of Show, Venue Tech-Spec, and Vendor/Rental COI tools to Production section
</commit_message>
<xml_diff>
--- a/Revital_Service_Pricing_Draft.xlsx
+++ b/Revital_Service_Pricing_Draft.xlsx
@@ -22,9 +22,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="142">
-  <si>
-    <t xml:space="preserve">Draft starting prices, researched from small-business/local-agency market benchmarks (July 2026). Edit the yellow Suggested Price / Suggested Cost cells to your own numbers, then enter the final values into the Hub's Service Pricing Admin tool. Margin recalculates automatically.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="144">
+  <si>
+    <t xml:space="preserve">Draft starting prices, researched from small-business/local-agency market benchmarks (July 2026). Edit the yellow Suggested Price / Suggested Cost cells to your own numbers, then enter the final values into the Hub's Service Pricing Admin tool. Margin recalculates automatically. Cost estimate basis: HubSpot/Sprout/Klaviyo use real software costs; every other service uses an estimated cost of 30% of price (monthly/retainer services) or 40% of price (one-time setup projects) for labor/delivery time — the same assumption the Proposal Calculator itself falls back to when no real cost is set. Replace with actual contractor/time costs as you get real numbers.</t>
   </si>
   <si>
     <t xml:space="preserve">Category</t>
@@ -412,6 +412,12 @@
   </si>
   <si>
     <t xml:space="preserve">Sum of Suggested One-Time Setup Prices ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum of Suggested Cost ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overall Margin (%)</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -454,9 +460,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -599,7 +606,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -648,11 +655,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -927,7 +942,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -975,11 +990,11 @@
         <v>350</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">D4-E4</f>
-        <v>350</v>
+        <v>245</v>
       </c>
       <c r="G4" s="3"/>
     </row>
@@ -997,11 +1012,11 @@
         <v>400</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">D5-E5</f>
-        <v>400</v>
+        <v>280</v>
       </c>
       <c r="G5" s="3"/>
     </row>
@@ -1019,11 +1034,11 @@
         <v>150</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">D6-E6</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G6" s="3"/>
     </row>
@@ -1041,11 +1056,11 @@
         <v>250</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">D7-E7</f>
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="G7" s="3"/>
     </row>
@@ -1063,11 +1078,11 @@
         <v>200</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">D8-E8</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G8" s="3"/>
     </row>
@@ -1085,11 +1100,11 @@
         <v>100</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">D9-E9</f>
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G9" s="3"/>
     </row>
@@ -1107,11 +1122,11 @@
         <v>100</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">D10-E10</f>
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G10" s="3"/>
     </row>
@@ -1129,11 +1144,11 @@
         <v>150</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">D11-E11</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G11" s="3"/>
     </row>
@@ -1151,11 +1166,11 @@
         <v>600</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="F12" s="8" t="n">
         <f aca="false">D12-E12</f>
-        <v>600</v>
+        <v>420</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>20</v>
@@ -1175,11 +1190,11 @@
         <v>500</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F13" s="8" t="n">
         <f aca="false">D13-E13</f>
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>20</v>
@@ -1199,11 +1214,11 @@
         <v>600</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="F14" s="8" t="n">
         <f aca="false">D14-E14</f>
-        <v>600</v>
+        <v>420</v>
       </c>
       <c r="G14" s="6" t="s">
         <v>20</v>
@@ -1223,11 +1238,11 @@
         <v>350</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="F15" s="8" t="n">
         <f aca="false">D15-E15</f>
-        <v>350</v>
+        <v>245</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>20</v>
@@ -1247,11 +1262,11 @@
         <v>350</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="F16" s="8" t="n">
         <f aca="false">D16-E16</f>
-        <v>350</v>
+        <v>245</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>20</v>
@@ -1271,11 +1286,11 @@
         <v>200</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F17" s="8" t="n">
         <f aca="false">D17-E17</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G17" s="6"/>
     </row>
@@ -1293,11 +1308,11 @@
         <v>300</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F18" s="8" t="n">
         <f aca="false">D18-E18</f>
-        <v>300</v>
+        <v>210</v>
       </c>
       <c r="G18" s="6"/>
     </row>
@@ -1315,11 +1330,11 @@
         <v>500</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F19" s="8" t="n">
         <f aca="false">D19-E19</f>
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G19" s="6"/>
     </row>
@@ -1337,11 +1352,11 @@
         <v>150</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F20" s="8" t="n">
         <f aca="false">D20-E20</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G20" s="6"/>
     </row>
@@ -1359,11 +1374,11 @@
         <v>250</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F21" s="8" t="n">
         <f aca="false">D21-E21</f>
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="G21" s="6"/>
     </row>
@@ -1381,11 +1396,11 @@
         <v>150</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F22" s="8" t="n">
         <f aca="false">D22-E22</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G22" s="6"/>
     </row>
@@ -1403,11 +1418,11 @@
         <v>700</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="F23" s="5" t="n">
         <f aca="false">D23-E23</f>
-        <v>700</v>
+        <v>490</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>20</v>
@@ -1427,11 +1442,11 @@
         <v>500</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F24" s="5" t="n">
         <f aca="false">D24-E24</f>
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>20</v>
@@ -1451,11 +1466,11 @@
         <v>600</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="F25" s="5" t="n">
         <f aca="false">D25-E25</f>
-        <v>600</v>
+        <v>420</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>20</v>
@@ -1475,11 +1490,11 @@
         <v>500</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F26" s="5" t="n">
         <f aca="false">D26-E26</f>
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>20</v>
@@ -1499,11 +1514,11 @@
         <v>200</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F27" s="5" t="n">
         <f aca="false">D27-E27</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G27" s="3"/>
     </row>
@@ -1521,11 +1536,11 @@
         <v>200</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F28" s="5" t="n">
         <f aca="false">D28-E28</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G28" s="3"/>
     </row>
@@ -1543,11 +1558,11 @@
         <v>150</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F29" s="5" t="n">
         <f aca="false">D29-E29</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G29" s="3"/>
     </row>
@@ -1565,11 +1580,11 @@
         <v>200</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F30" s="5" t="n">
         <f aca="false">D30-E30</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G30" s="3"/>
     </row>
@@ -1587,11 +1602,11 @@
         <v>350</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="F31" s="5" t="n">
         <f aca="false">D31-E31</f>
-        <v>350</v>
+        <v>210</v>
       </c>
       <c r="G31" s="3"/>
     </row>
@@ -1609,11 +1624,11 @@
         <v>150</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F32" s="5" t="n">
         <f aca="false">D32-E32</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G32" s="3"/>
     </row>
@@ -1631,11 +1646,11 @@
         <v>400</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F33" s="8" t="n">
         <f aca="false">D33-E33</f>
-        <v>400</v>
+        <v>280</v>
       </c>
       <c r="G33" s="6"/>
     </row>
@@ -1653,11 +1668,11 @@
         <v>350</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="F34" s="8" t="n">
         <f aca="false">D34-E34</f>
-        <v>350</v>
+        <v>245</v>
       </c>
       <c r="G34" s="6"/>
     </row>
@@ -1675,11 +1690,11 @@
         <v>450</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="F35" s="8" t="n">
         <f aca="false">D35-E35</f>
-        <v>450</v>
+        <v>315</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>47</v>
@@ -1699,11 +1714,11 @@
         <v>400</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F36" s="8" t="n">
         <f aca="false">D36-E36</f>
-        <v>400</v>
+        <v>280</v>
       </c>
       <c r="G36" s="6"/>
     </row>
@@ -1721,11 +1736,11 @@
         <v>200</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F37" s="8" t="n">
         <f aca="false">D37-E37</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G37" s="6"/>
     </row>
@@ -1743,11 +1758,11 @@
         <v>350</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="F38" s="8" t="n">
         <f aca="false">D38-E38</f>
-        <v>350</v>
+        <v>245</v>
       </c>
       <c r="G38" s="6"/>
     </row>
@@ -1765,11 +1780,11 @@
         <v>500</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F39" s="8" t="n">
         <f aca="false">D39-E39</f>
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G39" s="6"/>
     </row>
@@ -1787,11 +1802,11 @@
         <v>150</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F40" s="8" t="n">
         <f aca="false">D40-E40</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G40" s="6"/>
     </row>
@@ -1809,11 +1824,11 @@
         <v>150</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F41" s="8" t="n">
         <f aca="false">D41-E41</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G41" s="6"/>
     </row>
@@ -1831,11 +1846,11 @@
         <v>250</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F42" s="5" t="n">
         <f aca="false">D42-E42</f>
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="G42" s="3"/>
     </row>
@@ -1853,11 +1868,11 @@
         <v>200</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F43" s="5" t="n">
         <f aca="false">D43-E43</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G43" s="3"/>
     </row>
@@ -1875,11 +1890,11 @@
         <v>300</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F44" s="5" t="n">
         <f aca="false">D44-E44</f>
-        <v>300</v>
+        <v>210</v>
       </c>
       <c r="G44" s="3"/>
     </row>
@@ -1897,11 +1912,11 @@
         <v>150</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F45" s="5" t="n">
         <f aca="false">D45-E45</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G45" s="3"/>
     </row>
@@ -1919,11 +1934,11 @@
         <v>200</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F46" s="5" t="n">
         <f aca="false">D46-E46</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G46" s="3"/>
     </row>
@@ -1941,11 +1956,11 @@
         <v>300</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F47" s="5" t="n">
         <f aca="false">D47-E47</f>
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="G47" s="3"/>
     </row>
@@ -1963,11 +1978,11 @@
         <v>150</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F48" s="5" t="n">
         <f aca="false">D48-E48</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G48" s="3"/>
     </row>
@@ -1985,11 +2000,11 @@
         <v>200</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F49" s="5" t="n">
         <f aca="false">D49-E49</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G49" s="3"/>
     </row>
@@ -2007,11 +2022,11 @@
         <v>250</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F50" s="5" t="n">
         <f aca="false">D50-E50</f>
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="G50" s="3"/>
     </row>
@@ -2029,11 +2044,11 @@
         <v>100</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F51" s="5" t="n">
         <f aca="false">D51-E51</f>
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G51" s="3"/>
     </row>
@@ -2051,11 +2066,11 @@
         <v>400</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="F52" s="5" t="n">
         <f aca="false">D52-E52</f>
-        <v>400</v>
+        <v>240</v>
       </c>
       <c r="G52" s="3"/>
     </row>
@@ -2073,11 +2088,11 @@
         <v>100</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F53" s="5" t="n">
         <f aca="false">D53-E53</f>
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G53" s="3"/>
     </row>
@@ -2095,11 +2110,11 @@
         <v>3500</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="F54" s="8" t="n">
         <f aca="false">D54-E54</f>
-        <v>3500</v>
+        <v>2100</v>
       </c>
       <c r="G54" s="6"/>
     </row>
@@ -2117,11 +2132,11 @@
         <v>500</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F55" s="8" t="n">
         <f aca="false">D55-E55</f>
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="G55" s="6" t="s">
         <v>70</v>
@@ -2141,11 +2156,11 @@
         <v>600</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="F56" s="8" t="n">
         <f aca="false">D56-E56</f>
-        <v>600</v>
+        <v>360</v>
       </c>
       <c r="G56" s="6"/>
     </row>
@@ -2163,11 +2178,11 @@
         <v>150</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F57" s="8" t="n">
         <f aca="false">D57-E57</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G57" s="6"/>
     </row>
@@ -2185,11 +2200,11 @@
         <v>300</v>
       </c>
       <c r="E58" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F58" s="8" t="n">
         <f aca="false">D58-E58</f>
-        <v>300</v>
+        <v>210</v>
       </c>
       <c r="G58" s="6"/>
     </row>
@@ -2207,11 +2222,11 @@
         <v>300</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F59" s="8" t="n">
         <f aca="false">D59-E59</f>
-        <v>300</v>
+        <v>210</v>
       </c>
       <c r="G59" s="6"/>
     </row>
@@ -2229,11 +2244,11 @@
         <v>200</v>
       </c>
       <c r="E60" s="7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F60" s="8" t="n">
         <f aca="false">D60-E60</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G60" s="6"/>
     </row>
@@ -2251,11 +2266,11 @@
         <v>150</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F61" s="8" t="n">
         <f aca="false">D61-E61</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G61" s="6"/>
     </row>
@@ -2273,11 +2288,11 @@
         <v>50</v>
       </c>
       <c r="E62" s="7" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F62" s="8" t="n">
         <f aca="false">D62-E62</f>
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="G62" s="6" t="s">
         <v>78</v>
@@ -2297,11 +2312,11 @@
         <v>300</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F63" s="8" t="n">
         <f aca="false">D63-E63</f>
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="G63" s="6"/>
     </row>
@@ -2319,11 +2334,11 @@
         <v>800</v>
       </c>
       <c r="E64" s="7" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="F64" s="8" t="n">
         <f aca="false">D64-E64</f>
-        <v>800</v>
+        <v>480</v>
       </c>
       <c r="G64" s="6"/>
     </row>
@@ -2341,11 +2356,11 @@
         <v>150</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F65" s="8" t="n">
         <f aca="false">D65-E65</f>
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="G65" s="6"/>
     </row>
@@ -2363,11 +2378,11 @@
         <v>500</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F66" s="5" t="n">
         <f aca="false">D66-E66</f>
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G66" s="3"/>
     </row>
@@ -2385,11 +2400,11 @@
         <v>300</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F67" s="5" t="n">
         <f aca="false">D67-E67</f>
-        <v>300</v>
+        <v>210</v>
       </c>
       <c r="G67" s="3"/>
     </row>
@@ -2407,11 +2422,11 @@
         <v>400</v>
       </c>
       <c r="E68" s="4" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="F68" s="5" t="n">
         <f aca="false">D68-E68</f>
-        <v>400</v>
+        <v>240</v>
       </c>
       <c r="G68" s="3"/>
     </row>
@@ -2429,11 +2444,11 @@
         <v>250</v>
       </c>
       <c r="E69" s="4" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F69" s="5" t="n">
         <f aca="false">D69-E69</f>
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="G69" s="3"/>
     </row>
@@ -2451,11 +2466,11 @@
         <v>200</v>
       </c>
       <c r="E70" s="4" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F70" s="5" t="n">
         <f aca="false">D70-E70</f>
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="G70" s="3"/>
     </row>
@@ -2473,11 +2488,11 @@
         <v>800</v>
       </c>
       <c r="E71" s="4" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="F71" s="5" t="n">
         <f aca="false">D71-E71</f>
-        <v>800</v>
+        <v>480</v>
       </c>
       <c r="G71" s="3"/>
     </row>
@@ -2495,11 +2510,11 @@
         <v>100</v>
       </c>
       <c r="E72" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F72" s="5" t="n">
         <f aca="false">D72-E72</f>
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G72" s="3"/>
     </row>
@@ -2517,11 +2532,11 @@
         <v>200</v>
       </c>
       <c r="E73" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F73" s="5" t="n">
         <f aca="false">D73-E73</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G73" s="3"/>
     </row>
@@ -2539,11 +2554,11 @@
         <v>300</v>
       </c>
       <c r="E74" s="4" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F74" s="5" t="n">
         <f aca="false">D74-E74</f>
-        <v>300</v>
+        <v>210</v>
       </c>
       <c r="G74" s="3"/>
     </row>
@@ -2561,11 +2576,11 @@
         <v>600</v>
       </c>
       <c r="E75" s="4" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="F75" s="5" t="n">
         <f aca="false">D75-E75</f>
-        <v>600</v>
+        <v>360</v>
       </c>
       <c r="G75" s="3"/>
     </row>
@@ -2583,11 +2598,11 @@
         <v>600</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="F76" s="8" t="n">
         <f aca="false">D76-E76</f>
-        <v>600</v>
+        <v>360</v>
       </c>
       <c r="G76" s="6" t="s">
         <v>95</v>
@@ -2607,11 +2622,11 @@
         <v>250</v>
       </c>
       <c r="E77" s="7" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F77" s="8" t="n">
         <f aca="false">D77-E77</f>
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="G77" s="6"/>
     </row>
@@ -2629,11 +2644,11 @@
         <v>400</v>
       </c>
       <c r="E78" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F78" s="8" t="n">
         <f aca="false">D78-E78</f>
-        <v>400</v>
+        <v>280</v>
       </c>
       <c r="G78" s="6"/>
     </row>
@@ -2651,11 +2666,11 @@
         <v>500</v>
       </c>
       <c r="E79" s="7" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F79" s="8" t="n">
         <f aca="false">D79-E79</f>
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="G79" s="6"/>
     </row>
@@ -2673,11 +2688,11 @@
         <v>300</v>
       </c>
       <c r="E80" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F80" s="8" t="n">
         <f aca="false">D80-E80</f>
-        <v>300</v>
+        <v>210</v>
       </c>
       <c r="G80" s="6"/>
     </row>
@@ -2695,11 +2710,11 @@
         <v>300</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F81" s="8" t="n">
         <f aca="false">D81-E81</f>
-        <v>300</v>
+        <v>210</v>
       </c>
       <c r="G81" s="6"/>
     </row>
@@ -2717,11 +2732,11 @@
         <v>400</v>
       </c>
       <c r="E82" s="7" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="F82" s="8" t="n">
         <f aca="false">D82-E82</f>
-        <v>400</v>
+        <v>240</v>
       </c>
       <c r="G82" s="6"/>
     </row>
@@ -2739,11 +2754,11 @@
         <v>200</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F83" s="8" t="n">
         <f aca="false">D83-E83</f>
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G83" s="6"/>
     </row>
@@ -2761,11 +2776,11 @@
         <v>500</v>
       </c>
       <c r="E84" s="7" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F84" s="8" t="n">
         <f aca="false">D84-E84</f>
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G84" s="6"/>
     </row>
@@ -2783,11 +2798,11 @@
         <v>250</v>
       </c>
       <c r="E85" s="7" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F85" s="8" t="n">
         <f aca="false">D85-E85</f>
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="G85" s="6"/>
     </row>
@@ -2877,11 +2892,11 @@
         <v>300</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F89" s="8" t="n">
         <f aca="false">D89-E89</f>
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>114</v>
@@ -2901,11 +2916,11 @@
         <v>600</v>
       </c>
       <c r="E90" s="7" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="F90" s="8" t="n">
         <f aca="false">D90-E90</f>
-        <v>600</v>
+        <v>360</v>
       </c>
       <c r="G90" s="6" t="s">
         <v>116</v>
@@ -2925,11 +2940,11 @@
         <v>250</v>
       </c>
       <c r="E91" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F91" s="8" t="n">
         <f aca="false">D91-E91</f>
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="G91" s="6" t="s">
         <v>118</v>
@@ -2949,11 +2964,11 @@
         <v>200</v>
       </c>
       <c r="E92" s="7" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F92" s="8" t="n">
         <f aca="false">D92-E92</f>
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="G92" s="6"/>
     </row>
@@ -2971,11 +2986,11 @@
         <v>400</v>
       </c>
       <c r="E93" s="7" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="F93" s="8" t="n">
         <f aca="false">D93-E93</f>
-        <v>400</v>
+        <v>240</v>
       </c>
       <c r="G93" s="6" t="s">
         <v>121</v>
@@ -2995,11 +3010,11 @@
         <v>150</v>
       </c>
       <c r="E94" s="7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F94" s="8" t="n">
         <f aca="false">D94-E94</f>
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="G94" s="6" t="s">
         <v>123</v>
@@ -3019,11 +3034,11 @@
         <v>300</v>
       </c>
       <c r="E95" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F95" s="8" t="n">
         <f aca="false">D95-E95</f>
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="G95" s="6" t="s">
         <v>125</v>
@@ -3043,11 +3058,11 @@
         <v>150</v>
       </c>
       <c r="E96" s="7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F96" s="8" t="n">
         <f aca="false">D96-E96</f>
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="G96" s="6"/>
     </row>
@@ -3070,13 +3085,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3092,6 +3109,12 @@
       <c r="D1" s="9" t="s">
         <v>129</v>
       </c>
+      <c r="E1" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
@@ -3109,6 +3132,14 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A2,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>0</v>
       </c>
+      <c r="E2" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A2,'Price Sheet'!E:E)</f>
+        <v>510</v>
+      </c>
+      <c r="F2" s="12" t="n">
+        <f aca="false">IFERROR((C2+D2-E2)/(C2+D2),"—")</f>
+        <v>0.7</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
@@ -3126,6 +3157,14 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A3,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>500</v>
       </c>
+      <c r="E3" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A3,'Price Sheet'!E:E)</f>
+        <v>1235</v>
+      </c>
+      <c r="F3" s="12" t="n">
+        <f aca="false">IFERROR((C3+D3-E3)/(C3+D3),"—")</f>
+        <v>0.687341772151899</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
@@ -3143,6 +3182,14 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A4,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>350</v>
       </c>
+      <c r="E4" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A4,'Price Sheet'!E:E)</f>
+        <v>1100</v>
+      </c>
+      <c r="F4" s="12" t="n">
+        <f aca="false">IFERROR((C4+D4-E4)/(C4+D4),"—")</f>
+        <v>0.690140845070423</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
@@ -3160,6 +3207,14 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A5,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>500</v>
       </c>
+      <c r="E5" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A5,'Price Sheet'!E:E)</f>
+        <v>935</v>
+      </c>
+      <c r="F5" s="12" t="n">
+        <f aca="false">IFERROR((C5+D5-E5)/(C5+D5),"—")</f>
+        <v>0.683050847457627</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
@@ -3177,6 +3232,14 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A6,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>700</v>
       </c>
+      <c r="E6" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A6,'Price Sheet'!E:E)</f>
+        <v>850</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <f aca="false">IFERROR((C6+D6-E6)/(C6+D6),"—")</f>
+        <v>0.673076923076923</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
@@ -3194,6 +3257,14 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A7,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>5200</v>
       </c>
+      <c r="E7" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A7,'Price Sheet'!E:E)</f>
+        <v>2620</v>
+      </c>
+      <c r="F7" s="12" t="n">
+        <f aca="false">IFERROR((C7+D7-E7)/(C7+D7),"—")</f>
+        <v>0.625714285714286</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
@@ -3211,6 +3282,14 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A8,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>2500</v>
       </c>
+      <c r="E8" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A8,'Price Sheet'!E:E)</f>
+        <v>1345</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <f aca="false">IFERROR((C8+D8-E8)/(C8+D8),"—")</f>
+        <v>0.631506849315069</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
@@ -3228,6 +3307,14 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A9,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>1500</v>
       </c>
+      <c r="E9" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A9,'Price Sheet'!E:E)</f>
+        <v>1260</v>
+      </c>
+      <c r="F9" s="12" t="n">
+        <f aca="false">IFERROR((C9+D9-E9)/(C9+D9),"—")</f>
+        <v>0.65945945945946</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
@@ -3245,6 +3332,14 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A10,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>0</v>
       </c>
+      <c r="E10" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A10,'Price Sheet'!E:E)</f>
+        <v>294</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <f aca="false">IFERROR((C10+D10-E10)/(C10+D10),"—")</f>
+        <v>0.244215938303342</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
@@ -3262,22 +3357,38 @@
         <f aca="false">SUMIFS('Price Sheet'!D:D,'Price Sheet'!A:A,A11,'Price Sheet'!C:C,"One-Time Setup")</f>
         <v>2350</v>
       </c>
+      <c r="E11" s="11" t="n">
+        <f aca="false">SUMIF('Price Sheet'!A:A,A11,'Price Sheet'!E:E)</f>
+        <v>940</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <f aca="false">IFERROR((C11+D11-E11)/(C11+D11),"—")</f>
+        <v>0.6</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="B12" s="12" t="n">
+      <c r="A12" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="13" t="n">
         <f aca="false">SUM(B2:B11)</f>
         <v>93</v>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="14" t="n">
         <f aca="false">SUM(C2:C11)</f>
         <v>18239</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">SUM(D2:D11)</f>
         <v>13600</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <f aca="false">SUM(E2:E11)</f>
+        <v>11089</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <f aca="false">IFERROR((C12+D12-E12)/(C12+D12),"—")</f>
+        <v>0.651716448380917</v>
       </c>
     </row>
   </sheetData>
@@ -3303,58 +3414,58 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>131</v>
+      <c r="A1" s="16" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
-        <v>132</v>
+      <c r="A3" s="17" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>133</v>
+      <c r="A4" s="17" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
-        <v>134</v>
+      <c r="A5" s="17" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>135</v>
+      <c r="A6" s="17" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>136</v>
+      <c r="A7" s="17" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
-        <v>137</v>
+      <c r="A8" s="17" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
-        <v>138</v>
+      <c r="A9" s="17" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>139</v>
+      <c r="A10" s="17" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
-        <v>140</v>
+      <c r="A11" s="17" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>141</v>
+      <c r="A12" s="17" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>